<commit_message>
docs: DEVELOPER.md — 6 reguł z sesji 2026-03-15/16 (id=72)
</commit_message>
<xml_diff>
--- a/solutions/bi/TraElem/TraElem_plan.xlsx
+++ b/solutions/bi/TraElem/TraElem_plan.xlsx
@@ -2310,22 +2310,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kalkulacja_VAT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CASE: N=Od netto, B=Od brutto, ELSE Nieznane(val)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Techniczny flag sposobu kalkulacji - nie dla uzytkownikow BI</t>
+          <t>Sposob kalkulacji VAT na pozycji</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Ilosc x cena = wartosc (flag techniczny)</t>
+          <t>Ilosc x cena = wartosc (flag)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3315,22 +3315,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rowna_IloscxCena</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CASE: 0=Nieaktywne, 1=Aktywne, ELSE Nieznane(val)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Techniczny flag kalkulacji</t>
+          <t>Czy na pozycji obowiazuje rownanie ilosc*cena=wartosc</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Wartosci walutowe od ksiegowych (flag)</t>
+          <t>Wartosci walutowe od ksiegowych</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3356,22 +3356,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Wartosci_Od_Ksiegowych</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CASE: 0=Nie, 1=Tak, ELSE Nieznane(val)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Techniczny flag kalkulacji</t>
+          <t>Czy wartosci walutowe sa liczone od wartosci ksiegowych</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>

</xml_diff>